<commit_message>
added the excel file devices
</commit_message>
<xml_diff>
--- a/inventory/devices.xlsx
+++ b/inventory/devices.xlsx
@@ -5,15 +5,15 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prajwal\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prajwal\Documents\NetOpsAutomationSuite\inventory\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{458A131B-35DD-4903-A015-6F3F037C0293}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{183910F7-47F2-411E-B5D7-4ED4EBC4822B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9FAE7D83-CE1D-4413-AFEE-730678F908ED}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="88">
   <si>
     <t>Status</t>
   </si>
@@ -36,9 +36,6 @@
     <t>Hostname</t>
   </si>
   <si>
-    <t>Management IP</t>
-  </si>
-  <si>
     <t>Category</t>
   </si>
   <si>
@@ -48,21 +45,9 @@
     <t>Vendor</t>
   </si>
   <si>
-    <t>Credential Profile</t>
-  </si>
-  <si>
     <t>Active</t>
   </si>
   <si>
-    <t>NY</t>
-  </si>
-  <si>
-    <t>RTR01</t>
-  </si>
-  <si>
-    <t>10.10.10.1</t>
-  </si>
-  <si>
     <t>Router</t>
   </si>
   <si>
@@ -75,41 +60,243 @@
     <t>TACACS</t>
   </si>
   <si>
-    <t>SW01</t>
-  </si>
-  <si>
-    <t>10.10.10.2</t>
-  </si>
-  <si>
     <t>Switch</t>
   </si>
   <si>
     <t>IOS_SWITCH</t>
   </si>
   <si>
-    <t>CEDGE01</t>
-  </si>
-  <si>
-    <t>10.10.10.3</t>
-  </si>
-  <si>
     <t>CEDGE</t>
+  </si>
+  <si>
+    <t>Management_IP</t>
+  </si>
+  <si>
+    <t>Platform</t>
+  </si>
+  <si>
+    <t>OS</t>
+  </si>
+  <si>
+    <t>Credential_Profile</t>
+  </si>
+  <si>
+    <t>AB</t>
+  </si>
+  <si>
+    <t>AB-RTR01</t>
+  </si>
+  <si>
+    <t>192.168.10.1</t>
+  </si>
+  <si>
+    <t>ISR4331</t>
+  </si>
+  <si>
+    <t>IOS-XE</t>
+  </si>
+  <si>
+    <t>AB-CEDGE01</t>
+  </si>
+  <si>
+    <t>192.168.10.2</t>
+  </si>
+  <si>
+    <t>Catalyst 8300</t>
+  </si>
+  <si>
+    <t>IOS-XE SD-WAN</t>
+  </si>
+  <si>
+    <t>AB-VEDGE01</t>
+  </si>
+  <si>
+    <t>192.168.10.3</t>
+  </si>
+  <si>
+    <t>VEDGE</t>
+  </si>
+  <si>
+    <t>vEdge Cloud</t>
+  </si>
+  <si>
+    <t>Viptela</t>
+  </si>
+  <si>
+    <t>AB-SW01</t>
+  </si>
+  <si>
+    <t>192.168.10.11</t>
+  </si>
+  <si>
+    <t>Catalyst 9300</t>
+  </si>
+  <si>
+    <t>AB-SW02</t>
+  </si>
+  <si>
+    <t>192.168.10.12</t>
+  </si>
+  <si>
+    <t>Catalyst 9200</t>
+  </si>
+  <si>
+    <t>AB-WLC01</t>
+  </si>
+  <si>
+    <t>192.168.10.20</t>
+  </si>
+  <si>
+    <t>Wireless</t>
+  </si>
+  <si>
+    <t>AIREOS_WLC</t>
+  </si>
+  <si>
+    <t>5520 WLC</t>
+  </si>
+  <si>
+    <t>AireOS</t>
+  </si>
+  <si>
+    <t>WLC_ADMIN</t>
+  </si>
+  <si>
+    <t>AB-AP01</t>
+  </si>
+  <si>
+    <t>192.168.10.30</t>
+  </si>
+  <si>
+    <t>Access Point</t>
+  </si>
+  <si>
+    <t>AP</t>
+  </si>
+  <si>
+    <t>Catalyst 9130</t>
+  </si>
+  <si>
+    <t>AC</t>
+  </si>
+  <si>
+    <t>AC-RTR01</t>
+  </si>
+  <si>
+    <t>192.168.20.1</t>
+  </si>
+  <si>
+    <t>ISR4451</t>
+  </si>
+  <si>
+    <t>AC-CEDGE01</t>
+  </si>
+  <si>
+    <t>192.168.20.2</t>
+  </si>
+  <si>
+    <t>Catalyst 8500</t>
+  </si>
+  <si>
+    <t>AC-SW01</t>
+  </si>
+  <si>
+    <t>192.168.20.11</t>
+  </si>
+  <si>
+    <t>AC-WLC01</t>
+  </si>
+  <si>
+    <t>192.168.20.20</t>
+  </si>
+  <si>
+    <t>9800-L</t>
+  </si>
+  <si>
+    <t>AD</t>
+  </si>
+  <si>
+    <t>AD-RTR01</t>
+  </si>
+  <si>
+    <t>192.168.30.1</t>
+  </si>
+  <si>
+    <t>ISR4321</t>
+  </si>
+  <si>
+    <t>AD-VEDGE01</t>
+  </si>
+  <si>
+    <t>192.168.30.2</t>
+  </si>
+  <si>
+    <t>vEdge 1000</t>
+  </si>
+  <si>
+    <t>AD-SW01</t>
+  </si>
+  <si>
+    <t>192.168.30.11</t>
+  </si>
+  <si>
+    <t>AD-WLC01</t>
+  </si>
+  <si>
+    <t>192.168.30.20</t>
+  </si>
+  <si>
+    <t>Disabled</t>
+  </si>
+  <si>
+    <t>AE</t>
+  </si>
+  <si>
+    <t>AE-RTR01</t>
+  </si>
+  <si>
+    <t>192.168.40.1</t>
+  </si>
+  <si>
+    <t>AE-SW01</t>
+  </si>
+  <si>
+    <t>192.168.40.11</t>
+  </si>
+  <si>
+    <t>AF</t>
+  </si>
+  <si>
+    <t>AF-RTR01</t>
+  </si>
+  <si>
+    <t>192.168.50.1</t>
+  </si>
+  <si>
+    <t>ISR4431</t>
+  </si>
+  <si>
+    <t>AF-SW01</t>
+  </si>
+  <si>
+    <t>192.168.50.11</t>
+  </si>
+  <si>
+    <t>AF-WLC01</t>
+  </si>
+  <si>
+    <t>192.168.50.20</t>
+  </si>
+  <si>
+    <t>9800-CL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -125,7 +312,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -133,35 +320,14 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -476,22 +642,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1C15FBD-B047-4ABE-A6C3-21021A42EA89}">
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultColWidth="20.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB166A4E-274D-4F26-ABEE-B2E2BCFC0F24}">
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="20.44140625" style="2"/>
+    <col min="1" max="1" width="7.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -502,97 +670,665 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+      <c r="F2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="3" t="s">
+      <c r="G2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+      <c r="G10" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+      <c r="G13" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F17" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" s="3" t="s">
+      <c r="G17" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="H17" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G18" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="H18" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>15</v>
+      <c r="I18" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added soome test devices eveng
</commit_message>
<xml_diff>
--- a/inventory/devices.xlsx
+++ b/inventory/devices.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prajwal\Documents\NetOpsAutomationSuite\inventory\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F0FFEC4-0594-4E2A-9BF9-A3DEC421D0D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F445C29-D8B9-4977-BAEE-EBD26B4DDB07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9FAE7D83-CE1D-4413-AFEE-730678F908ED}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{9FAE7D83-CE1D-4413-AFEE-730678F908ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$2:$J$21</definedName>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="97">
   <si>
     <t>Status</t>
   </si>
@@ -289,14 +290,52 @@
   </si>
   <si>
     <t>AUTOMATION</t>
+  </si>
+  <si>
+    <t>LAB</t>
+  </si>
+  <si>
+    <t>LAB-RTR01</t>
+  </si>
+  <si>
+    <t>IOSv</t>
+  </si>
+  <si>
+    <t>IOS</t>
+  </si>
+  <si>
+    <t>LAB-L3SW01</t>
+  </si>
+  <si>
+    <t>IOSvL2</t>
+  </si>
+  <si>
+    <t>LAB-L2SW01</t>
+  </si>
+  <si>
+    <t>10.234.29.150</t>
+  </si>
+  <si>
+    <t>10.234.29.151</t>
+  </si>
+  <si>
+    <t>10.234.29.152</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -312,7 +351,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -320,15 +359,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1324,4 +1380,142 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D802F4D-80F2-47F1-87DC-19DC44FAD1CD}">
+  <dimension ref="A1:J4"/>
+  <sheetFormatPr defaultColWidth="18.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
added the Bat file
</commit_message>
<xml_diff>
--- a/inventory/devices.xlsx
+++ b/inventory/devices.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prajwal\Documents\Projects\NetOpsAutomationSuite\inventory\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A7998F0-FA26-46B8-82D2-B5AA60B757C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C74AFF4C-A8EE-40D4-A257-A2C8F966780C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9FAE7D83-CE1D-4413-AFEE-730678F908ED}"/>
   </bookViews>
@@ -99,13 +99,13 @@
     <t>LAN-SW</t>
   </si>
   <si>
-    <t>192.168.123.2</t>
-  </si>
-  <si>
-    <t>172.28.139.200</t>
-  </si>
-  <si>
-    <t>192.168.122.2</t>
+    <t>10.161.44.200</t>
+  </si>
+  <si>
+    <t>10.161.44.201</t>
+  </si>
+  <si>
+    <t>10.161.44.202</t>
   </si>
 </sst>
 </file>
@@ -528,7 +528,7 @@
         <v>21</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>7</v>
@@ -560,7 +560,7 @@
         <v>22</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>10</v>
@@ -592,7 +592,7 @@
         <v>23</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>10</v>

</xml_diff>